<commit_message>
Refresh fourth 18 October workbook revision with independent local QA
</commit_message>
<xml_diff>
--- a/Weekly_Leadership_Source_Workbook.xlsx
+++ b/Weekly_Leadership_Source_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmoreno\Documents\Project References\US IT Network Projects\IT Program Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6C96F71F-C7E8-4C0A-BE71-B0FDE5681EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{157C5C0C-0511-490D-AC8E-9B0D25332A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IT Security" sheetId="2" r:id="rId1"/>
@@ -3265,9 +3265,6 @@
     <t>IT Infrastructure Update email, 14-Oct-2026 PST; IT Network Team Meeting Notes, 16-Oct-2026 PST.</t>
   </si>
   <si>
-    <t>Tenant Wi-Fi PPSK and VLAN Governance</t>
-  </si>
-  <si>
     <t>Technical pattern tested / ownership, approval, lifecycle, and isolation validation pending</t>
   </si>
   <si>
@@ -3283,9 +3280,6 @@
     <t>Jerimar to share the configuration standard. Assign the service owner and approver; define who creates, distributes, stores, rotates, revokes, and audits keys; verify tenant-to-VLAN mapping, firewall policy, cross-tenant isolation, same-tenant behavior, logging, onboarding/offboarding, and support. Conduct a controlled validation and retain results.</t>
   </si>
   <si>
-    <t>Jerimar Castaneda / QBerg-Qbert Team / Network Engineering / Security / Tenant Operations / Robert Moreno</t>
-  </si>
-  <si>
     <t>Unclear key ownership or unverified isolation can cause unauthorized tenant access, credential leakage, inconsistent offboarding, and audit gaps.</t>
   </si>
   <si>
@@ -3692,6 +3686,12 @@
   </si>
   <si>
     <t>Mel Gutierrez / Robert Moreno / Mike Wang's replacement pending / Robotics Team</t>
+  </si>
+  <si>
+    <t>Tenant Wi-Fi and VLAN Governance</t>
+  </si>
+  <si>
+    <t>Jerimar Castaneda / Cubework IT Installation Team / Network Engineering / Security / Tenant Operations / Robert Moreno</t>
   </si>
 </sst>
 </file>
@@ -6925,7 +6925,7 @@
         <v>650</v>
       </c>
       <c r="K2" s="51" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="L2" s="51" t="s">
         <v>651</v>
@@ -6934,7 +6934,7 @@
         <v>652</v>
       </c>
       <c r="N2" s="56" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="160" customHeight="1">
@@ -6969,7 +6969,7 @@
         <v>657</v>
       </c>
       <c r="K3" s="51" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="L3" s="51" t="s">
         <v>658</v>
@@ -6978,7 +6978,7 @@
         <v>659</v>
       </c>
       <c r="N3" s="56" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="160" customHeight="1">
@@ -7013,7 +7013,7 @@
         <v>664</v>
       </c>
       <c r="K4" s="51" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="L4" s="51" t="s">
         <v>665</v>
@@ -7022,7 +7022,7 @@
         <v>666</v>
       </c>
       <c r="N4" s="56" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="39.65" customHeight="1">
@@ -7057,7 +7057,7 @@
         <v>24</v>
       </c>
       <c r="K5" s="8" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="L5" s="8" t="s">
         <v>25</v>
@@ -7229,7 +7229,7 @@
         <v>48</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="L10" s="12" t="s">
         <v>49</v>
@@ -10242,10 +10242,10 @@
         <v>64</v>
       </c>
       <c r="B64" s="46" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C64" s="46" t="s">
         <v>1020</v>
-      </c>
-      <c r="C64" s="46" t="s">
-        <v>1021</v>
       </c>
       <c r="D64" s="116" t="s">
         <v>13</v>
@@ -10254,31 +10254,31 @@
         <v>1001</v>
       </c>
       <c r="F64" s="47" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="G64" s="48">
         <v>0.7</v>
       </c>
       <c r="H64" s="49" t="s">
+        <v>1022</v>
+      </c>
+      <c r="I64" s="49" t="s">
         <v>1023</v>
       </c>
-      <c r="I64" s="49" t="s">
+      <c r="J64" s="49" t="s">
         <v>1024</v>
       </c>
-      <c r="J64" s="49" t="s">
+      <c r="K64" s="49" t="s">
+        <v>1162</v>
+      </c>
+      <c r="L64" s="49" t="s">
         <v>1025</v>
       </c>
-      <c r="K64" s="49" t="s">
+      <c r="M64" s="49" t="s">
         <v>1026</v>
       </c>
-      <c r="L64" s="49" t="s">
+      <c r="N64" s="49" t="s">
         <v>1027</v>
-      </c>
-      <c r="M64" s="49" t="s">
-        <v>1028</v>
-      </c>
-      <c r="N64" s="49" t="s">
-        <v>1029</v>
       </c>
     </row>
   </sheetData>
@@ -11072,22 +11072,22 @@
         <v>207</v>
       </c>
       <c r="I2" s="30" t="s">
-        <v>1030</v>
+        <v>1028</v>
       </c>
       <c r="J2" s="30" t="s">
-        <v>1031</v>
+        <v>1029</v>
       </c>
       <c r="K2" s="30" t="s">
         <v>208</v>
       </c>
       <c r="L2" s="30" t="s">
+        <v>1030</v>
+      </c>
+      <c r="M2" s="30" t="s">
+        <v>1031</v>
+      </c>
+      <c r="N2" s="30" t="s">
         <v>1032</v>
-      </c>
-      <c r="M2" s="30" t="s">
-        <v>1033</v>
-      </c>
-      <c r="N2" s="30" t="s">
-        <v>1034</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="43.5">
@@ -11116,22 +11116,22 @@
         <v>211</v>
       </c>
       <c r="I3" s="30" t="s">
-        <v>1035</v>
+        <v>1033</v>
       </c>
       <c r="J3" s="30" t="s">
-        <v>1036</v>
+        <v>1034</v>
       </c>
       <c r="K3" s="30" t="s">
         <v>208</v>
       </c>
       <c r="L3" s="30" t="s">
+        <v>1035</v>
+      </c>
+      <c r="M3" s="30" t="s">
+        <v>1036</v>
+      </c>
+      <c r="N3" s="30" t="s">
         <v>1037</v>
-      </c>
-      <c r="M3" s="30" t="s">
-        <v>1038</v>
-      </c>
-      <c r="N3" s="30" t="s">
-        <v>1039</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="43.5">
@@ -11248,22 +11248,22 @@
         <v>221</v>
       </c>
       <c r="I6" s="30" t="s">
-        <v>1040</v>
+        <v>1038</v>
       </c>
       <c r="J6" s="30" t="s">
-        <v>1041</v>
+        <v>1039</v>
       </c>
       <c r="K6" s="30" t="s">
         <v>214</v>
       </c>
       <c r="L6" s="30" t="s">
+        <v>1040</v>
+      </c>
+      <c r="M6" s="30" t="s">
+        <v>1041</v>
+      </c>
+      <c r="N6" s="30" t="s">
         <v>1042</v>
-      </c>
-      <c r="M6" s="30" t="s">
-        <v>1043</v>
-      </c>
-      <c r="N6" s="30" t="s">
-        <v>1044</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="29">
@@ -11359,7 +11359,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="30" t="s">
-        <v>1045</v>
+        <v>1043</v>
       </c>
       <c r="C9" s="29" t="s">
         <v>17</v>
@@ -11377,25 +11377,25 @@
         <v>0.3</v>
       </c>
       <c r="H9" s="30" t="s">
+        <v>1044</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>1045</v>
+      </c>
+      <c r="J9" s="30" t="s">
         <v>1046</v>
-      </c>
-      <c r="I9" s="30" t="s">
-        <v>1047</v>
-      </c>
-      <c r="J9" s="30" t="s">
-        <v>1048</v>
       </c>
       <c r="K9" s="30" t="s">
         <v>208</v>
       </c>
       <c r="L9" s="30" t="s">
+        <v>1047</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>1048</v>
+      </c>
+      <c r="N9" s="30" t="s">
         <v>1049</v>
-      </c>
-      <c r="M9" s="30" t="s">
-        <v>1050</v>
-      </c>
-      <c r="N9" s="30" t="s">
-        <v>1051</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="87">
@@ -11403,7 +11403,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="30" t="s">
-        <v>1052</v>
+        <v>1050</v>
       </c>
       <c r="C10" s="29" t="s">
         <v>17</v>
@@ -11421,25 +11421,25 @@
         <v>0.2</v>
       </c>
       <c r="H10" s="30" t="s">
+        <v>1051</v>
+      </c>
+      <c r="I10" s="30" t="s">
+        <v>1052</v>
+      </c>
+      <c r="J10" s="30" t="s">
         <v>1053</v>
-      </c>
-      <c r="I10" s="30" t="s">
-        <v>1054</v>
-      </c>
-      <c r="J10" s="30" t="s">
-        <v>1055</v>
       </c>
       <c r="K10" s="30" t="s">
         <v>214</v>
       </c>
       <c r="L10" s="30" t="s">
+        <v>1054</v>
+      </c>
+      <c r="M10" s="30" t="s">
+        <v>1055</v>
+      </c>
+      <c r="N10" s="30" t="s">
         <v>1056</v>
-      </c>
-      <c r="M10" s="30" t="s">
-        <v>1057</v>
-      </c>
-      <c r="N10" s="30" t="s">
-        <v>1058</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -11729,7 +11729,7 @@
         <v>247</v>
       </c>
       <c r="C4" s="37" t="s">
-        <v>1112</v>
+        <v>1110</v>
       </c>
       <c r="D4" s="130" t="s">
         <v>13</v>
@@ -11738,31 +11738,31 @@
         <v>46303</v>
       </c>
       <c r="F4" s="40" t="s">
-        <v>1113</v>
+        <v>1111</v>
       </c>
       <c r="G4" s="128">
         <v>0.75</v>
       </c>
       <c r="H4" s="38" t="s">
+        <v>1112</v>
+      </c>
+      <c r="I4" s="38" t="s">
+        <v>1113</v>
+      </c>
+      <c r="J4" s="38" t="s">
         <v>1114</v>
       </c>
-      <c r="I4" s="38" t="s">
+      <c r="K4" s="38" t="s">
         <v>1115</v>
       </c>
-      <c r="J4" s="38" t="s">
+      <c r="L4" s="38" t="s">
         <v>1116</v>
       </c>
-      <c r="K4" s="38" t="s">
+      <c r="M4" s="38" t="s">
         <v>1117</v>
       </c>
-      <c r="L4" s="38" t="s">
+      <c r="N4" s="131" t="s">
         <v>1118</v>
-      </c>
-      <c r="M4" s="38" t="s">
-        <v>1119</v>
-      </c>
-      <c r="N4" s="131" t="s">
-        <v>1120</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="116" customHeight="1">
@@ -11773,7 +11773,7 @@
         <v>248</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="D5" s="132" t="s">
         <v>506</v>
@@ -11782,31 +11782,31 @@
         <v>46240</v>
       </c>
       <c r="F5" s="40" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="G5" s="128">
         <v>0.4</v>
       </c>
       <c r="H5" s="38" t="s">
+        <v>1121</v>
+      </c>
+      <c r="I5" s="38" t="s">
+        <v>1122</v>
+      </c>
+      <c r="J5" s="38" t="s">
         <v>1123</v>
       </c>
-      <c r="I5" s="38" t="s">
+      <c r="K5" s="38" t="s">
         <v>1124</v>
       </c>
-      <c r="J5" s="38" t="s">
+      <c r="L5" s="38" t="s">
         <v>1125</v>
       </c>
-      <c r="K5" s="38" t="s">
+      <c r="M5" s="38" t="s">
         <v>1126</v>
       </c>
-      <c r="L5" s="38" t="s">
+      <c r="N5" s="129" t="s">
         <v>1127</v>
-      </c>
-      <c r="M5" s="38" t="s">
-        <v>1128</v>
-      </c>
-      <c r="N5" s="129" t="s">
-        <v>1129</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="174">
@@ -11817,7 +11817,7 @@
         <v>249</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="D6" s="133" t="s">
         <v>13</v>
@@ -11826,31 +11826,31 @@
         <v>514</v>
       </c>
       <c r="F6" s="40" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="G6" s="128">
         <v>0.7</v>
       </c>
       <c r="H6" s="38" t="s">
+        <v>1130</v>
+      </c>
+      <c r="I6" s="38" t="s">
+        <v>1131</v>
+      </c>
+      <c r="J6" s="38" t="s">
         <v>1132</v>
       </c>
-      <c r="I6" s="38" t="s">
+      <c r="K6" s="38" t="s">
         <v>1133</v>
       </c>
-      <c r="J6" s="38" t="s">
+      <c r="L6" s="38" t="s">
         <v>1134</v>
       </c>
-      <c r="K6" s="38" t="s">
+      <c r="M6" s="38" t="s">
         <v>1135</v>
       </c>
-      <c r="L6" s="38" t="s">
+      <c r="N6" s="131" t="s">
         <v>1136</v>
-      </c>
-      <c r="M6" s="38" t="s">
-        <v>1137</v>
-      </c>
-      <c r="N6" s="131" t="s">
-        <v>1138</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="72.5">
@@ -11905,7 +11905,7 @@
         <v>258</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="D8" s="125" t="s">
         <v>21</v>
@@ -11914,31 +11914,31 @@
         <v>46188</v>
       </c>
       <c r="F8" s="40" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="G8" s="128">
         <v>0.8</v>
       </c>
       <c r="H8" s="38" t="s">
+        <v>1139</v>
+      </c>
+      <c r="I8" s="38" t="s">
+        <v>1140</v>
+      </c>
+      <c r="J8" s="38" t="s">
         <v>1141</v>
       </c>
-      <c r="I8" s="38" t="s">
+      <c r="K8" s="38" t="s">
         <v>1142</v>
       </c>
-      <c r="J8" s="38" t="s">
+      <c r="L8" s="38" t="s">
         <v>1143</v>
       </c>
-      <c r="K8" s="38" t="s">
+      <c r="M8" s="38" t="s">
         <v>1144</v>
       </c>
-      <c r="L8" s="38" t="s">
+      <c r="N8" s="131" t="s">
         <v>1145</v>
-      </c>
-      <c r="M8" s="38" t="s">
-        <v>1146</v>
-      </c>
-      <c r="N8" s="131" t="s">
-        <v>1147</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="188.5">
@@ -11949,7 +11949,7 @@
         <v>547</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="D9" s="133" t="s">
         <v>13</v>
@@ -11958,31 +11958,31 @@
         <v>548</v>
       </c>
       <c r="F9" s="40" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="G9" s="128">
         <v>0.7</v>
       </c>
       <c r="H9" s="38" t="s">
+        <v>1148</v>
+      </c>
+      <c r="I9" s="38" t="s">
+        <v>1149</v>
+      </c>
+      <c r="J9" s="38" t="s">
         <v>1150</v>
       </c>
-      <c r="I9" s="38" t="s">
+      <c r="K9" s="38" t="s">
         <v>1151</v>
       </c>
-      <c r="J9" s="38" t="s">
+      <c r="L9" s="38" t="s">
         <v>1152</v>
       </c>
-      <c r="K9" s="38" t="s">
+      <c r="M9" s="38" t="s">
         <v>1153</v>
       </c>
-      <c r="L9" s="38" t="s">
+      <c r="N9" s="134" t="s">
         <v>1154</v>
-      </c>
-      <c r="M9" s="38" t="s">
-        <v>1155</v>
-      </c>
-      <c r="N9" s="134" t="s">
-        <v>1156</v>
       </c>
     </row>
   </sheetData>
@@ -13266,7 +13266,7 @@
         <v>318</v>
       </c>
       <c r="C2" s="96" t="s">
-        <v>1059</v>
+        <v>1057</v>
       </c>
       <c r="D2" s="122" t="s">
         <v>21</v>
@@ -13284,22 +13284,22 @@
         <v>319</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>1060</v>
+        <v>1058</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>1061</v>
+        <v>1059</v>
       </c>
       <c r="K2" s="5" t="s">
         <v>320</v>
       </c>
       <c r="L2" s="5" t="s">
+        <v>1060</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>1061</v>
+      </c>
+      <c r="N2" s="5" t="s">
         <v>1062</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>1063</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>1064</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="78" customHeight="1">
@@ -13310,7 +13310,7 @@
         <v>321</v>
       </c>
       <c r="C3" s="96" t="s">
-        <v>1065</v>
+        <v>1063</v>
       </c>
       <c r="D3" s="122" t="s">
         <v>21</v>
@@ -13328,22 +13328,22 @@
         <v>322</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>1066</v>
+        <v>1064</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>1067</v>
+        <v>1065</v>
       </c>
       <c r="K3" s="5" t="s">
         <v>323</v>
       </c>
       <c r="L3" s="5" t="s">
+        <v>1066</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>1067</v>
+      </c>
+      <c r="N3" s="5" t="s">
         <v>1068</v>
-      </c>
-      <c r="M3" s="5" t="s">
-        <v>1069</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>1070</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="78" customHeight="1">
@@ -13398,7 +13398,7 @@
         <v>332</v>
       </c>
       <c r="C5" s="123" t="s">
-        <v>1071</v>
+        <v>1069</v>
       </c>
       <c r="D5" s="122" t="s">
         <v>21</v>
@@ -13416,22 +13416,22 @@
         <v>516</v>
       </c>
       <c r="I5" s="5" t="s">
+        <v>1070</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>1071</v>
+      </c>
+      <c r="K5" s="5" t="s">
         <v>1072</v>
       </c>
-      <c r="J5" s="5" t="s">
+      <c r="L5" s="5" t="s">
         <v>1073</v>
       </c>
-      <c r="K5" s="5" t="s">
+      <c r="M5" s="5" t="s">
         <v>1074</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="N5" s="5" t="s">
         <v>1075</v>
-      </c>
-      <c r="M5" s="5" t="s">
-        <v>1076</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>1077</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="96" customHeight="1">
@@ -13442,7 +13442,7 @@
         <v>333</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>1078</v>
+        <v>1076</v>
       </c>
       <c r="D6" s="122" t="s">
         <v>21</v>
@@ -13451,31 +13451,31 @@
         <v>334</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>1079</v>
+        <v>1077</v>
       </c>
       <c r="G6" s="14">
         <v>0.98347107438016534</v>
       </c>
       <c r="H6" s="12" t="s">
+        <v>1078</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>1079</v>
+      </c>
+      <c r="J6" s="12" t="s">
         <v>1080</v>
       </c>
-      <c r="I6" s="12" t="s">
+      <c r="K6" s="12" t="s">
         <v>1081</v>
       </c>
-      <c r="J6" s="12" t="s">
+      <c r="L6" s="12" t="s">
         <v>1082</v>
       </c>
-      <c r="K6" s="12" t="s">
+      <c r="M6" s="12" t="s">
         <v>1083</v>
       </c>
-      <c r="L6" s="12" t="s">
+      <c r="N6" s="12" t="s">
         <v>1084</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>1085</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>1086</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="78" customHeight="1">
@@ -13662,7 +13662,7 @@
         <v>369</v>
       </c>
       <c r="C11" s="96" t="s">
-        <v>1087</v>
+        <v>1085</v>
       </c>
       <c r="D11" s="122" t="s">
         <v>21</v>
@@ -13680,22 +13680,22 @@
         <v>518</v>
       </c>
       <c r="I11" s="5" t="s">
+        <v>1086</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>1087</v>
+      </c>
+      <c r="K11" s="5" t="s">
         <v>1088</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="L11" s="5" t="s">
         <v>1089</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="M11" s="5" t="s">
         <v>1090</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="N11" s="5" t="s">
         <v>1091</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>1092</v>
-      </c>
-      <c r="N11" s="5" t="s">
-        <v>1093</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="78" customHeight="1">
@@ -13794,7 +13794,7 @@
         <v>528</v>
       </c>
       <c r="C14" s="96" t="s">
-        <v>1094</v>
+        <v>1092</v>
       </c>
       <c r="D14" s="122" t="s">
         <v>21</v>
@@ -13803,7 +13803,7 @@
         <v>159</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>1095</v>
+        <v>1093</v>
       </c>
       <c r="G14" s="14">
         <v>0.98347107438016534</v>
@@ -13812,22 +13812,22 @@
         <v>529</v>
       </c>
       <c r="I14" s="12" t="s">
+        <v>1094</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>1095</v>
+      </c>
+      <c r="K14" s="12" t="s">
         <v>1096</v>
       </c>
-      <c r="J14" s="12" t="s">
+      <c r="L14" s="12" t="s">
         <v>1097</v>
       </c>
-      <c r="K14" s="12" t="s">
+      <c r="M14" s="12" t="s">
         <v>1098</v>
       </c>
-      <c r="L14" s="12" t="s">
+      <c r="N14" s="12" t="s">
         <v>1099</v>
-      </c>
-      <c r="M14" s="12" t="s">
-        <v>1100</v>
-      </c>
-      <c r="N14" s="12" t="s">
-        <v>1101</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="112.5">
@@ -13835,10 +13835,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>1102</v>
+        <v>1100</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>1103</v>
+        <v>1101</v>
       </c>
       <c r="D15" s="124" t="s">
         <v>13</v>
@@ -13847,31 +13847,31 @@
         <v>46296</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>1104</v>
+        <v>1102</v>
       </c>
       <c r="G15" s="14">
         <v>0.7</v>
       </c>
       <c r="H15" s="12" t="s">
+        <v>1103</v>
+      </c>
+      <c r="I15" s="12" t="s">
+        <v>1104</v>
+      </c>
+      <c r="J15" s="12" t="s">
         <v>1105</v>
       </c>
-      <c r="I15" s="12" t="s">
+      <c r="K15" s="12" t="s">
         <v>1106</v>
       </c>
-      <c r="J15" s="12" t="s">
+      <c r="L15" s="12" t="s">
         <v>1107</v>
       </c>
-      <c r="K15" s="12" t="s">
+      <c r="M15" s="12" t="s">
         <v>1108</v>
       </c>
-      <c r="L15" s="12" t="s">
+      <c r="N15" s="12" t="s">
         <v>1109</v>
-      </c>
-      <c r="M15" s="12" t="s">
-        <v>1110</v>
-      </c>
-      <c r="N15" s="12" t="s">
-        <v>1111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh IT and Technology branding and preserve original workbook filename
</commit_message>
<xml_diff>
--- a/Weekly_Leadership_Source_Workbook.xlsx
+++ b/Weekly_Leadership_Source_Workbook.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmoreno\Documents\Project References\US IT Network Projects\IT Program Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4ADABBCB-83A2-4C49-AC30-BE40FC6E2892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{93F753A3-D275-4A0B-9FF4-3532B6199207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5352,6 +5352,214 @@
       </fill>
     </dxf>
     <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -6204,214 +6412,6 @@
         </bottom>
       </border>
     </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color indexed="64"/>
-        </left>
-        <right style="thin">
-          <color indexed="64"/>
-        </right>
-        <top style="thin">
-          <color indexed="64"/>
-        </top>
-        <bottom style="thin">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -6488,19 +6488,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A71A1BB0-309E-488F-B49F-600E48896486}" name="TeamRoadmapTable1" displayName="TeamRoadmapTable1" ref="A1:M7" totalsRowShown="0">
   <autoFilter ref="A1:M7" xr:uid="{A71A1BB0-309E-488F-B49F-600E48896486}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{C980970C-B48D-4335-A7E5-7AA2F6802A24}" name="#" dataDxfId="122"/>
-    <tableColumn id="2" xr3:uid="{96D6F9DD-6A4C-4A23-8A2B-F5291F35F77B}" name="Project / Workstream" dataDxfId="121"/>
-    <tableColumn id="3" xr3:uid="{888D9B81-A395-47DF-80CE-DA1131D1376F}" name="Status" dataDxfId="120"/>
-    <tableColumn id="4" xr3:uid="{CD231B59-4E25-4B82-A1EB-E707CA38F7F6}" name="Start Date" dataDxfId="119"/>
-    <tableColumn id="5" xr3:uid="{09DB588B-E2A0-4761-85A9-73F0AAB8C56E}" name="Completion Date" dataDxfId="118"/>
-    <tableColumn id="6" xr3:uid="{1A4661DA-45C5-46A1-916F-2F7D6E08BB15}" name="% of Completion" dataDxfId="117"/>
-    <tableColumn id="7" xr3:uid="{48DEBC38-3245-436F-B70F-5021B1121FE5}" name="Core Objective" dataDxfId="116"/>
-    <tableColumn id="8" xr3:uid="{290E8003-D7B1-4D5D-857D-CBB894CC223E}" name="Current Progress" dataDxfId="115"/>
-    <tableColumn id="9" xr3:uid="{BCACD256-A4F8-499C-BFD0-C1A9A8DABF38}" name="Key Next Steps" dataDxfId="114"/>
-    <tableColumn id="10" xr3:uid="{5A660B4D-1115-4650-BF44-269E14C2F4B6}" name="Owners / Direct Responsible Individual" dataDxfId="113"/>
-    <tableColumn id="11" xr3:uid="{8A1FC045-4525-484D-851C-CE33F806003F}" name="Key Risks / Blockers" dataDxfId="112"/>
-    <tableColumn id="12" xr3:uid="{FF19E1D6-D997-457B-AED2-186127759682}" name="Management Attention" dataDxfId="111"/>
-    <tableColumn id="13" xr3:uid="{7B618D71-AE79-4B84-AB4E-BE24031BD242}" name="Source / Notes" dataDxfId="110"/>
+    <tableColumn id="1" xr3:uid="{C980970C-B48D-4335-A7E5-7AA2F6802A24}" name="#" dataDxfId="135"/>
+    <tableColumn id="2" xr3:uid="{96D6F9DD-6A4C-4A23-8A2B-F5291F35F77B}" name="Project / Workstream" dataDxfId="134"/>
+    <tableColumn id="3" xr3:uid="{888D9B81-A395-47DF-80CE-DA1131D1376F}" name="Status" dataDxfId="133"/>
+    <tableColumn id="4" xr3:uid="{CD231B59-4E25-4B82-A1EB-E707CA38F7F6}" name="Start Date" dataDxfId="132"/>
+    <tableColumn id="5" xr3:uid="{09DB588B-E2A0-4761-85A9-73F0AAB8C56E}" name="Completion Date" dataDxfId="131"/>
+    <tableColumn id="6" xr3:uid="{1A4661DA-45C5-46A1-916F-2F7D6E08BB15}" name="% of Completion" dataDxfId="130"/>
+    <tableColumn id="7" xr3:uid="{48DEBC38-3245-436F-B70F-5021B1121FE5}" name="Core Objective" dataDxfId="129"/>
+    <tableColumn id="8" xr3:uid="{290E8003-D7B1-4D5D-857D-CBB894CC223E}" name="Current Progress" dataDxfId="128"/>
+    <tableColumn id="9" xr3:uid="{BCACD256-A4F8-499C-BFD0-C1A9A8DABF38}" name="Key Next Steps" dataDxfId="127"/>
+    <tableColumn id="10" xr3:uid="{5A660B4D-1115-4650-BF44-269E14C2F4B6}" name="Owners / Direct Responsible Individual" dataDxfId="126"/>
+    <tableColumn id="11" xr3:uid="{8A1FC045-4525-484D-851C-CE33F806003F}" name="Key Risks / Blockers" dataDxfId="125"/>
+    <tableColumn id="12" xr3:uid="{FF19E1D6-D997-457B-AED2-186127759682}" name="Management Attention" dataDxfId="124"/>
+    <tableColumn id="13" xr3:uid="{7B618D71-AE79-4B84-AB4E-BE24031BD242}" name="Source / Notes" dataDxfId="123"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6510,19 +6510,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{3A043A57-0A20-4E85-A933-3BB0CB08E4C9}" name="TeamRoadmapTable2" displayName="TeamRoadmapTable2" ref="A1:M19" totalsRowShown="0">
   <autoFilter ref="A1:M19" xr:uid="{3A043A57-0A20-4E85-A933-3BB0CB08E4C9}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{04D2C9D7-4A63-4D43-8460-5BA1E57998E1}" name="#" dataDxfId="109"/>
-    <tableColumn id="2" xr3:uid="{DE32A74B-ACED-4731-9D8E-7226F401412D}" name="Project / Workstream" dataDxfId="108"/>
-    <tableColumn id="3" xr3:uid="{04149982-9EF5-449F-961A-BF0867C647C1}" name="Status" dataDxfId="107"/>
-    <tableColumn id="4" xr3:uid="{A1E93C6D-5D79-4BAD-8158-FC06AB9A0A2A}" name="Start Date" dataDxfId="106"/>
-    <tableColumn id="5" xr3:uid="{9D70E4F2-14E3-4514-82F7-82857D4D498F}" name="Completion Date" dataDxfId="105"/>
-    <tableColumn id="6" xr3:uid="{DE2824DE-72CA-4C5B-B785-96216DFB725E}" name="% of Completion" dataDxfId="104"/>
-    <tableColumn id="7" xr3:uid="{0E7CE61A-FFCE-42EC-9A19-4DC35F7D82EC}" name="Core Objective" dataDxfId="103"/>
-    <tableColumn id="8" xr3:uid="{DA97804F-4A67-45F4-8DC4-109A8061E995}" name="Current Progress" dataDxfId="102"/>
-    <tableColumn id="9" xr3:uid="{3BA55CC0-9EA7-4EFE-BA4C-A10EF8069CDF}" name="Key Next Steps" dataDxfId="101"/>
-    <tableColumn id="10" xr3:uid="{F28926D7-580C-4F13-B486-AF82074B882E}" name="Owners / Direct Responsible Individual " dataDxfId="100"/>
-    <tableColumn id="11" xr3:uid="{7F73DD8A-CAFD-4606-9581-BD4E972F5D36}" name="Key Risks / Blockers" dataDxfId="99"/>
-    <tableColumn id="12" xr3:uid="{D7F0EE5A-FD00-467C-A756-3F85ED5C0E14}" name="Management Attention" dataDxfId="98"/>
-    <tableColumn id="13" xr3:uid="{28C61FA1-267E-4365-9DF4-7313CD4DA5E3}" name="Source / Notes" dataDxfId="97"/>
+    <tableColumn id="1" xr3:uid="{04D2C9D7-4A63-4D43-8460-5BA1E57998E1}" name="#" dataDxfId="122"/>
+    <tableColumn id="2" xr3:uid="{DE32A74B-ACED-4731-9D8E-7226F401412D}" name="Project / Workstream" dataDxfId="121"/>
+    <tableColumn id="3" xr3:uid="{04149982-9EF5-449F-961A-BF0867C647C1}" name="Status" dataDxfId="120"/>
+    <tableColumn id="4" xr3:uid="{A1E93C6D-5D79-4BAD-8158-FC06AB9A0A2A}" name="Start Date" dataDxfId="119"/>
+    <tableColumn id="5" xr3:uid="{9D70E4F2-14E3-4514-82F7-82857D4D498F}" name="Completion Date" dataDxfId="118"/>
+    <tableColumn id="6" xr3:uid="{DE2824DE-72CA-4C5B-B785-96216DFB725E}" name="% of Completion" dataDxfId="117"/>
+    <tableColumn id="7" xr3:uid="{0E7CE61A-FFCE-42EC-9A19-4DC35F7D82EC}" name="Core Objective" dataDxfId="116"/>
+    <tableColumn id="8" xr3:uid="{DA97804F-4A67-45F4-8DC4-109A8061E995}" name="Current Progress" dataDxfId="115"/>
+    <tableColumn id="9" xr3:uid="{3BA55CC0-9EA7-4EFE-BA4C-A10EF8069CDF}" name="Key Next Steps" dataDxfId="114"/>
+    <tableColumn id="10" xr3:uid="{F28926D7-580C-4F13-B486-AF82074B882E}" name="Owners / Direct Responsible Individual " dataDxfId="113"/>
+    <tableColumn id="11" xr3:uid="{7F73DD8A-CAFD-4606-9581-BD4E972F5D36}" name="Key Risks / Blockers" dataDxfId="112"/>
+    <tableColumn id="12" xr3:uid="{D7F0EE5A-FD00-467C-A756-3F85ED5C0E14}" name="Management Attention" dataDxfId="111"/>
+    <tableColumn id="13" xr3:uid="{28C61FA1-267E-4365-9DF4-7313CD4DA5E3}" name="Source / Notes" dataDxfId="110"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6532,13 +6532,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{43D12A05-4024-4190-889D-F8FEFB906ADF}" name="_10IoTTable" displayName="_10IoTTable" ref="A3:M7" totalsRowShown="0">
   <autoFilter ref="A3:M7" xr:uid="{43D12A05-4024-4190-889D-F8FEFB906ADF}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{9D1720D2-255E-4948-AEA4-87288BF22E61}" name="#" dataDxfId="96"/>
-    <tableColumn id="2" xr3:uid="{4CEBED98-D095-4FF0-AA5D-6905FADEA5E0}" name="Project / Workstream" dataDxfId="95"/>
-    <tableColumn id="3" xr3:uid="{E63C1969-65EA-4BA6-88C8-CDFA436DDC12}" name="Status" dataDxfId="94"/>
-    <tableColumn id="13" xr3:uid="{5C0468A9-CA1F-4BCC-9EFD-A6FE497EF0EA}" name="RAG Status" dataDxfId="93"/>
-    <tableColumn id="4" xr3:uid="{BD2A85DA-AC7D-412B-B2D3-E211E2A201B7}" name="Start Date" dataDxfId="92"/>
-    <tableColumn id="5" xr3:uid="{9D1F8663-B522-4F92-B037-83A09E5F1E2C}" name="Completion Date" dataDxfId="91"/>
-    <tableColumn id="6" xr3:uid="{9C8B4CFC-45ED-4D95-9EE8-678A45C388A2}" name="% of Completion" dataDxfId="90"/>
+    <tableColumn id="1" xr3:uid="{9D1720D2-255E-4948-AEA4-87288BF22E61}" name="#" dataDxfId="109"/>
+    <tableColumn id="2" xr3:uid="{4CEBED98-D095-4FF0-AA5D-6905FADEA5E0}" name="Project / Workstream" dataDxfId="108"/>
+    <tableColumn id="3" xr3:uid="{E63C1969-65EA-4BA6-88C8-CDFA436DDC12}" name="Status" dataDxfId="107"/>
+    <tableColumn id="13" xr3:uid="{5C0468A9-CA1F-4BCC-9EFD-A6FE497EF0EA}" name="RAG Status" dataDxfId="106"/>
+    <tableColumn id="4" xr3:uid="{BD2A85DA-AC7D-412B-B2D3-E211E2A201B7}" name="Start Date" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{9D1F8663-B522-4F92-B037-83A09E5F1E2C}" name="Completion Date" dataDxfId="104"/>
+    <tableColumn id="6" xr3:uid="{9C8B4CFC-45ED-4D95-9EE8-678A45C388A2}" name="% of Completion" dataDxfId="103"/>
     <tableColumn id="7" xr3:uid="{8042D65A-E9A7-440A-8DA3-E859E12CE7CC}" name="Core Objective"/>
     <tableColumn id="8" xr3:uid="{9DE2D962-3BBB-4A29-890B-C8C6BB038444}" name="Current Progress"/>
     <tableColumn id="9" xr3:uid="{684619BD-39A8-4E89-B9A3-C74834F32A8A}" name="Key Next Steps"/>
@@ -6551,23 +6551,23 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{1ECFDA90-66A0-4F30-B0FF-7E730E1479EF}" name="TeamRoadmapTable4" displayName="TeamRoadmapTable4" ref="A1:N10" totalsRowShown="0" headerRowDxfId="89" dataDxfId="88" dataCellStyle="常规">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{1ECFDA90-66A0-4F30-B0FF-7E730E1479EF}" name="TeamRoadmapTable4" displayName="TeamRoadmapTable4" ref="A1:N10" totalsRowShown="0" headerRowDxfId="102" dataDxfId="101" dataCellStyle="常规">
   <autoFilter ref="A1:N10" xr:uid="{1ECFDA90-66A0-4F30-B0FF-7E730E1479EF}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{679CF03B-1214-4CC0-9C0B-50F40DA8A237}" name="#" dataDxfId="87" dataCellStyle="常规"/>
-    <tableColumn id="2" xr3:uid="{190D03B6-3A2A-4849-8CD1-3CE10074EEFE}" name="Project / Workstream" dataDxfId="86" dataCellStyle="常规"/>
-    <tableColumn id="3" xr3:uid="{DF3A1391-53C9-42A8-9B4E-6E5AC03DE8CA}" name="Status" dataDxfId="85" dataCellStyle="常规"/>
-    <tableColumn id="15" xr3:uid="{A8F23B7A-2051-42FE-B1A7-F0B22DA7AEA3}" name="RAG Status" dataDxfId="84" dataCellStyle="常规"/>
-    <tableColumn id="4" xr3:uid="{FB882904-D83E-4AF4-94C7-D3D6C40D0A43}" name="Start Date" dataDxfId="83" dataCellStyle="常规"/>
-    <tableColumn id="5" xr3:uid="{F4997E23-B6A3-4C2E-A58C-B3F149E07E71}" name="Completion Date" dataDxfId="82" dataCellStyle="常规"/>
-    <tableColumn id="6" xr3:uid="{D21D1725-E004-4FA3-87DE-59FAC267E67C}" name="% of Completion" dataDxfId="81" dataCellStyle="常规"/>
-    <tableColumn id="7" xr3:uid="{85ECBED0-BAC5-4B91-8509-920E9DA6D49C}" name="Core Objective" dataDxfId="80" dataCellStyle="常规"/>
-    <tableColumn id="8" xr3:uid="{1BEF56B1-00D5-4AB9-80BA-54516FCD12F4}" name="Current Progress" dataDxfId="79" dataCellStyle="常规"/>
-    <tableColumn id="9" xr3:uid="{217482B5-A245-481C-BB74-5CCA909D64C7}" name="Key Next Steps" dataDxfId="78" dataCellStyle="常规"/>
-    <tableColumn id="10" xr3:uid="{99FB2831-B049-41B4-9630-30604A9C16D4}" name="Owners / Direct Responsible Individual" dataDxfId="77" dataCellStyle="常规"/>
-    <tableColumn id="11" xr3:uid="{96B9AD91-82DF-4634-9B78-C515E558FCD4}" name="Key Risks / Blockers" dataDxfId="76" dataCellStyle="常规"/>
-    <tableColumn id="12" xr3:uid="{37A3351C-8352-4160-8826-AF8B8E6368EF}" name="Management Attention" dataDxfId="75" dataCellStyle="常规"/>
-    <tableColumn id="13" xr3:uid="{7B16C62B-B1C1-471B-85DC-88990965CC5E}" name="Source / Notes" dataDxfId="74" dataCellStyle="常规"/>
+    <tableColumn id="1" xr3:uid="{679CF03B-1214-4CC0-9C0B-50F40DA8A237}" name="#" dataDxfId="100" dataCellStyle="常规"/>
+    <tableColumn id="2" xr3:uid="{190D03B6-3A2A-4849-8CD1-3CE10074EEFE}" name="Project / Workstream" dataDxfId="99" dataCellStyle="常规"/>
+    <tableColumn id="3" xr3:uid="{DF3A1391-53C9-42A8-9B4E-6E5AC03DE8CA}" name="Status" dataDxfId="98" dataCellStyle="常规"/>
+    <tableColumn id="15" xr3:uid="{A8F23B7A-2051-42FE-B1A7-F0B22DA7AEA3}" name="RAG Status" dataDxfId="97" dataCellStyle="常规"/>
+    <tableColumn id="4" xr3:uid="{FB882904-D83E-4AF4-94C7-D3D6C40D0A43}" name="Start Date" dataDxfId="96" dataCellStyle="常规"/>
+    <tableColumn id="5" xr3:uid="{F4997E23-B6A3-4C2E-A58C-B3F149E07E71}" name="Completion Date" dataDxfId="95" dataCellStyle="常规"/>
+    <tableColumn id="6" xr3:uid="{D21D1725-E004-4FA3-87DE-59FAC267E67C}" name="% of Completion" dataDxfId="94" dataCellStyle="常规"/>
+    <tableColumn id="7" xr3:uid="{85ECBED0-BAC5-4B91-8509-920E9DA6D49C}" name="Core Objective" dataDxfId="93" dataCellStyle="常规"/>
+    <tableColumn id="8" xr3:uid="{1BEF56B1-00D5-4AB9-80BA-54516FCD12F4}" name="Current Progress" dataDxfId="92" dataCellStyle="常规"/>
+    <tableColumn id="9" xr3:uid="{217482B5-A245-481C-BB74-5CCA909D64C7}" name="Key Next Steps" dataDxfId="91" dataCellStyle="常规"/>
+    <tableColumn id="10" xr3:uid="{99FB2831-B049-41B4-9630-30604A9C16D4}" name="Owners / Direct Responsible Individual" dataDxfId="90" dataCellStyle="常规"/>
+    <tableColumn id="11" xr3:uid="{96B9AD91-82DF-4634-9B78-C515E558FCD4}" name="Key Risks / Blockers" dataDxfId="89" dataCellStyle="常规"/>
+    <tableColumn id="12" xr3:uid="{37A3351C-8352-4160-8826-AF8B8E6368EF}" name="Management Attention" dataDxfId="88" dataCellStyle="常规"/>
+    <tableColumn id="13" xr3:uid="{7B16C62B-B1C1-471B-85DC-88990965CC5E}" name="Source / Notes" dataDxfId="87" dataCellStyle="常规"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6599,19 +6599,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AF29BE91-12F7-41D7-96DC-1435A4A1D6D5}" name="TeamRoadmapTable6" displayName="TeamRoadmapTable6" ref="A1:M12" totalsRowShown="0">
   <autoFilter ref="A1:M12" xr:uid="{AF29BE91-12F7-41D7-96DC-1435A4A1D6D5}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{D30BF4EC-955A-42A8-82DD-DFC1FA0E5E7D}" name="#" dataDxfId="135"/>
-    <tableColumn id="2" xr3:uid="{ED6809AB-855C-4EA2-9397-856F2BE4DAB5}" name="Project / Workstream" dataDxfId="134"/>
-    <tableColumn id="3" xr3:uid="{DEA9FC0A-0DA4-4864-B04F-5557D7CD8EE4}" name="Status" dataDxfId="133"/>
-    <tableColumn id="4" xr3:uid="{A47988CA-1547-453E-9F7C-2F040DF7A266}" name="Start Date" dataDxfId="132"/>
-    <tableColumn id="5" xr3:uid="{B2CE9BA8-8D83-4808-B5B6-1245DF87E76F}" name="Completion Date" dataDxfId="131"/>
-    <tableColumn id="6" xr3:uid="{7BA0FCD7-0715-4EFA-A1C9-7506AB98CF57}" name="% of Completion" dataDxfId="130"/>
-    <tableColumn id="7" xr3:uid="{7E29D23E-18DB-4895-8105-E582525A76DA}" name="Core Objective" dataDxfId="129"/>
-    <tableColumn id="8" xr3:uid="{B408C4DA-6CB0-428A-9D08-DD16AA355A61}" name="Current Progress" dataDxfId="128"/>
-    <tableColumn id="9" xr3:uid="{1DC2176A-256A-4A96-AD50-0B1E8B37A4A9}" name="Key Next Steps" dataDxfId="127"/>
-    <tableColumn id="10" xr3:uid="{06D17CEA-01D9-4ADD-B928-3449CB6F0519}" name="Owners / Direct Responsible Individual" dataDxfId="126"/>
-    <tableColumn id="11" xr3:uid="{AE5FD19A-866E-4462-85AB-0ED794227DC3}" name="Key Risks / Blockers" dataDxfId="125"/>
-    <tableColumn id="12" xr3:uid="{1ABD2D3B-AF76-4375-A3B2-7171D61620F4}" name="Management Attention" dataDxfId="124"/>
-    <tableColumn id="13" xr3:uid="{31BE1D2A-1D54-46BB-BD45-935CBF81148E}" name="Source / Notes" dataDxfId="123"/>
+    <tableColumn id="1" xr3:uid="{D30BF4EC-955A-42A8-82DD-DFC1FA0E5E7D}" name="#" dataDxfId="86"/>
+    <tableColumn id="2" xr3:uid="{ED6809AB-855C-4EA2-9397-856F2BE4DAB5}" name="Project / Workstream" dataDxfId="85"/>
+    <tableColumn id="3" xr3:uid="{DEA9FC0A-0DA4-4864-B04F-5557D7CD8EE4}" name="Status" dataDxfId="84"/>
+    <tableColumn id="4" xr3:uid="{A47988CA-1547-453E-9F7C-2F040DF7A266}" name="Start Date" dataDxfId="83"/>
+    <tableColumn id="5" xr3:uid="{B2CE9BA8-8D83-4808-B5B6-1245DF87E76F}" name="Completion Date" dataDxfId="82"/>
+    <tableColumn id="6" xr3:uid="{7BA0FCD7-0715-4EFA-A1C9-7506AB98CF57}" name="% of Completion" dataDxfId="81"/>
+    <tableColumn id="7" xr3:uid="{7E29D23E-18DB-4895-8105-E582525A76DA}" name="Core Objective" dataDxfId="80"/>
+    <tableColumn id="8" xr3:uid="{B408C4DA-6CB0-428A-9D08-DD16AA355A61}" name="Current Progress" dataDxfId="79"/>
+    <tableColumn id="9" xr3:uid="{1DC2176A-256A-4A96-AD50-0B1E8B37A4A9}" name="Key Next Steps" dataDxfId="78"/>
+    <tableColumn id="10" xr3:uid="{06D17CEA-01D9-4ADD-B928-3449CB6F0519}" name="Owners / Direct Responsible Individual" dataDxfId="77"/>
+    <tableColumn id="11" xr3:uid="{AE5FD19A-866E-4462-85AB-0ED794227DC3}" name="Key Risks / Blockers" dataDxfId="76"/>
+    <tableColumn id="12" xr3:uid="{1ABD2D3B-AF76-4375-A3B2-7171D61620F4}" name="Management Attention" dataDxfId="75"/>
+    <tableColumn id="13" xr3:uid="{31BE1D2A-1D54-46BB-BD45-935CBF81148E}" name="Source / Notes" dataDxfId="74"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Refresh latest 26 October attachment and verify source formatting semantics
</commit_message>
<xml_diff>
--- a/Weekly_Leadership_Source_Workbook.xlsx
+++ b/Weekly_Leadership_Source_Workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rmoreno\Documents\Project References\US IT Network Projects\IT Program Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5C38A7DD-E823-471A-9C55-061FC29BAF38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{70FFB88F-1F36-4E17-A158-454432839003}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IT Security" sheetId="2" r:id="rId1"/>
@@ -3010,14 +3010,14 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3025,7 +3025,29 @@
     <cellStyle name="Percent" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
     <cellStyle name="常规" xfId="1" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="147">
+  <dxfs count="129">
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b/>
@@ -3040,6 +3062,94 @@
     <dxf>
       <font>
         <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -3062,11 +3172,154 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF1F4E78"/>
+        <color rgb="FF9C0006"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFDDEBF7"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3084,11 +3337,11 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF9C0006"/>
+        <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3117,11 +3370,66 @@
     <dxf>
       <font>
         <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFE699"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF1F4E78"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3139,6 +3447,292 @@
     <dxf>
       <font>
         <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6E0B4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF1F4E78"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD9EAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF595959"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE7E6E6"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF1F4E78"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFD9EAF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF7F6000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -3161,6 +3755,28 @@
     <dxf>
       <font>
         <b/>
+        <color rgb="FF1F4E78"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDDEBF7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <color rgb="FF9C6500"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -3194,17 +3810,6 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -3216,814 +3821,11 @@
     <dxf>
       <font>
         <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
         <color rgb="FF9C6500"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF1F4E78"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDDEBF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF1F4E78"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFD9EAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF1F4E78"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFD9EAF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF7F6000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFE699"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF595959"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE7E6E6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF9C6500"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6E0B4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5014,19 +4816,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{A71A1BB0-309E-488F-B49F-600E48896486}" name="TeamRoadmapTable1" displayName="TeamRoadmapTable1" ref="A1:M7" totalsRowShown="0">
   <autoFilter ref="A1:M7" xr:uid="{A71A1BB0-309E-488F-B49F-600E48896486}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{C980970C-B48D-4335-A7E5-7AA2F6802A24}" name="#" dataDxfId="146"/>
-    <tableColumn id="2" xr3:uid="{96D6F9DD-6A4C-4A23-8A2B-F5291F35F77B}" name="Project / Workstream" dataDxfId="145"/>
-    <tableColumn id="3" xr3:uid="{888D9B81-A395-47DF-80CE-DA1131D1376F}" name="Status" dataDxfId="144"/>
-    <tableColumn id="4" xr3:uid="{CD231B59-4E25-4B82-A1EB-E707CA38F7F6}" name="Start Date" dataDxfId="143"/>
-    <tableColumn id="5" xr3:uid="{09DB588B-E2A0-4761-85A9-73F0AAB8C56E}" name="Completion Date" dataDxfId="142"/>
-    <tableColumn id="6" xr3:uid="{1A4661DA-45C5-46A1-916F-2F7D6E08BB15}" name="% of Completion" dataDxfId="141"/>
-    <tableColumn id="7" xr3:uid="{48DEBC38-3245-436F-B70F-5021B1121FE5}" name="Core Objective" dataDxfId="140"/>
-    <tableColumn id="8" xr3:uid="{290E8003-D7B1-4D5D-857D-CBB894CC223E}" name="Current Progress" dataDxfId="139"/>
-    <tableColumn id="9" xr3:uid="{BCACD256-A4F8-499C-BFD0-C1A9A8DABF38}" name="Key Next Steps" dataDxfId="138"/>
-    <tableColumn id="10" xr3:uid="{5A660B4D-1115-4650-BF44-269E14C2F4B6}" name="Owners / Direct Responsible Individual" dataDxfId="137"/>
-    <tableColumn id="11" xr3:uid="{8A1FC045-4525-484D-851C-CE33F806003F}" name="Key Risks / Blockers" dataDxfId="136"/>
-    <tableColumn id="12" xr3:uid="{FF19E1D6-D997-457B-AED2-186127759682}" name="Management Attention" dataDxfId="135"/>
-    <tableColumn id="13" xr3:uid="{7B618D71-AE79-4B84-AB4E-BE24031BD242}" name="Source / Notes" dataDxfId="134"/>
+    <tableColumn id="1" xr3:uid="{C980970C-B48D-4335-A7E5-7AA2F6802A24}" name="#" dataDxfId="128"/>
+    <tableColumn id="2" xr3:uid="{96D6F9DD-6A4C-4A23-8A2B-F5291F35F77B}" name="Project / Workstream" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{888D9B81-A395-47DF-80CE-DA1131D1376F}" name="Status" dataDxfId="126"/>
+    <tableColumn id="4" xr3:uid="{CD231B59-4E25-4B82-A1EB-E707CA38F7F6}" name="Start Date" dataDxfId="125"/>
+    <tableColumn id="5" xr3:uid="{09DB588B-E2A0-4761-85A9-73F0AAB8C56E}" name="Completion Date" dataDxfId="124"/>
+    <tableColumn id="6" xr3:uid="{1A4661DA-45C5-46A1-916F-2F7D6E08BB15}" name="% of Completion" dataDxfId="123"/>
+    <tableColumn id="7" xr3:uid="{48DEBC38-3245-436F-B70F-5021B1121FE5}" name="Core Objective" dataDxfId="122"/>
+    <tableColumn id="8" xr3:uid="{290E8003-D7B1-4D5D-857D-CBB894CC223E}" name="Current Progress" dataDxfId="121"/>
+    <tableColumn id="9" xr3:uid="{BCACD256-A4F8-499C-BFD0-C1A9A8DABF38}" name="Key Next Steps" dataDxfId="120"/>
+    <tableColumn id="10" xr3:uid="{5A660B4D-1115-4650-BF44-269E14C2F4B6}" name="Owners / Direct Responsible Individual" dataDxfId="119"/>
+    <tableColumn id="11" xr3:uid="{8A1FC045-4525-484D-851C-CE33F806003F}" name="Key Risks / Blockers" dataDxfId="118"/>
+    <tableColumn id="12" xr3:uid="{FF19E1D6-D997-457B-AED2-186127759682}" name="Management Attention" dataDxfId="117"/>
+    <tableColumn id="13" xr3:uid="{7B618D71-AE79-4B84-AB4E-BE24031BD242}" name="Source / Notes" dataDxfId="116"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5058,13 +4860,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{65DA8CF1-0749-447D-BE9F-234CC140F3D5}" name="_10IoTTable" displayName="_10IoTTable" ref="A3:M7" totalsRowShown="0">
   <autoFilter ref="A3:M7" xr:uid="{65DA8CF1-0749-447D-BE9F-234CC140F3D5}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{A42FBC5A-5AB7-4E56-8955-D33DD8B39A2F}" name="#" dataDxfId="133"/>
-    <tableColumn id="2" xr3:uid="{48895D70-CD40-454C-BCF6-E71E20E1B5D7}" name="Project / Workstream" dataDxfId="132"/>
-    <tableColumn id="3" xr3:uid="{7042EA98-2297-45CD-8FB8-4DB81434329B}" name="Status" dataDxfId="131"/>
-    <tableColumn id="13" xr3:uid="{6ACFE3C6-7C72-4612-B788-1A2EE239387D}" name="RAG Status" dataDxfId="130"/>
-    <tableColumn id="4" xr3:uid="{B077331C-655B-4625-B3AE-960E49A8DAA0}" name="Start Date" dataDxfId="129"/>
-    <tableColumn id="5" xr3:uid="{14C810B0-8C31-4BAC-B4AA-225493DA4C35}" name="Completion Date" dataDxfId="128"/>
-    <tableColumn id="6" xr3:uid="{92E2932C-BBDB-4580-9824-73C127586685}" name="% of Completion" dataDxfId="127"/>
+    <tableColumn id="1" xr3:uid="{A42FBC5A-5AB7-4E56-8955-D33DD8B39A2F}" name="#" dataDxfId="115"/>
+    <tableColumn id="2" xr3:uid="{48895D70-CD40-454C-BCF6-E71E20E1B5D7}" name="Project / Workstream" dataDxfId="114"/>
+    <tableColumn id="3" xr3:uid="{7042EA98-2297-45CD-8FB8-4DB81434329B}" name="Status" dataDxfId="113"/>
+    <tableColumn id="13" xr3:uid="{6ACFE3C6-7C72-4612-B788-1A2EE239387D}" name="RAG Status" dataDxfId="112"/>
+    <tableColumn id="4" xr3:uid="{B077331C-655B-4625-B3AE-960E49A8DAA0}" name="Start Date" dataDxfId="111"/>
+    <tableColumn id="5" xr3:uid="{14C810B0-8C31-4BAC-B4AA-225493DA4C35}" name="Completion Date" dataDxfId="110"/>
+    <tableColumn id="6" xr3:uid="{92E2932C-BBDB-4580-9824-73C127586685}" name="% of Completion" dataDxfId="109"/>
     <tableColumn id="7" xr3:uid="{637CBACF-931B-4A5D-83E3-D8F95A6B569E}" name="Core Objective"/>
     <tableColumn id="8" xr3:uid="{96183204-6BB9-41FA-A03C-6594655716D0}" name="Current Progress"/>
     <tableColumn id="9" xr3:uid="{761E254D-A73D-4E17-B889-C31A24AA6E25}" name="Key Next Steps"/>
@@ -5102,19 +4904,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{EFFD927E-694D-48DB-BDCB-B7EF17D92354}" name="TeamRoadmapTable6" displayName="TeamRoadmapTable6" ref="A1:M12" totalsRowShown="0">
   <autoFilter ref="A1:M12" xr:uid="{EFFD927E-694D-48DB-BDCB-B7EF17D92354}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{FD853018-9160-40B6-AD3A-01FBA01C8180}" name="#" dataDxfId="126"/>
-    <tableColumn id="2" xr3:uid="{1082E385-152B-497E-89DE-67429E70E855}" name="Project / Workstream" dataDxfId="125"/>
-    <tableColumn id="3" xr3:uid="{DD2D94DC-2FA3-4380-94F7-5B3B8DAB545E}" name="Status" dataDxfId="124"/>
-    <tableColumn id="4" xr3:uid="{90563E9B-C25F-4DAB-9B4B-10A06A29FF49}" name="Start Date" dataDxfId="123"/>
-    <tableColumn id="5" xr3:uid="{FAB56266-E4E8-457C-8294-2344A83E9AB5}" name="Completion Date" dataDxfId="122"/>
-    <tableColumn id="6" xr3:uid="{B5B770EA-2D63-4268-B956-B86A2D96D931}" name="% of Completion" dataDxfId="121"/>
-    <tableColumn id="7" xr3:uid="{9C244548-A355-4394-84DF-6C4F9C30B433}" name="Core Objective" dataDxfId="120"/>
-    <tableColumn id="8" xr3:uid="{49E7CA11-05AD-4974-9AEA-D42373D9A8C9}" name="Current Progress" dataDxfId="119"/>
-    <tableColumn id="9" xr3:uid="{33C40143-39AF-428C-BF9D-AD0CC8CF7C20}" name="Key Next Steps" dataDxfId="118"/>
-    <tableColumn id="10" xr3:uid="{171C6211-BEA3-4026-BB75-96BBCCB9F34F}" name="Owners / Direct Responsible Individual" dataDxfId="117"/>
-    <tableColumn id="11" xr3:uid="{52ABC80D-1F46-4C95-ADD7-573DD9895B58}" name="Key Risks / Blockers" dataDxfId="116"/>
-    <tableColumn id="12" xr3:uid="{71A740DB-BF55-484E-83A5-FB5F077091BA}" name="Management Attention" dataDxfId="115"/>
-    <tableColumn id="13" xr3:uid="{0BB4D142-9FDE-40BF-863F-DB4D20B001FC}" name="Source / Notes" dataDxfId="114"/>
+    <tableColumn id="1" xr3:uid="{FD853018-9160-40B6-AD3A-01FBA01C8180}" name="#" dataDxfId="108"/>
+    <tableColumn id="2" xr3:uid="{1082E385-152B-497E-89DE-67429E70E855}" name="Project / Workstream" dataDxfId="107"/>
+    <tableColumn id="3" xr3:uid="{DD2D94DC-2FA3-4380-94F7-5B3B8DAB545E}" name="Status" dataDxfId="106"/>
+    <tableColumn id="4" xr3:uid="{90563E9B-C25F-4DAB-9B4B-10A06A29FF49}" name="Start Date" dataDxfId="105"/>
+    <tableColumn id="5" xr3:uid="{FAB56266-E4E8-457C-8294-2344A83E9AB5}" name="Completion Date" dataDxfId="104"/>
+    <tableColumn id="6" xr3:uid="{B5B770EA-2D63-4268-B956-B86A2D96D931}" name="% of Completion" dataDxfId="103"/>
+    <tableColumn id="7" xr3:uid="{9C244548-A355-4394-84DF-6C4F9C30B433}" name="Core Objective" dataDxfId="102"/>
+    <tableColumn id="8" xr3:uid="{49E7CA11-05AD-4974-9AEA-D42373D9A8C9}" name="Current Progress" dataDxfId="101"/>
+    <tableColumn id="9" xr3:uid="{33C40143-39AF-428C-BF9D-AD0CC8CF7C20}" name="Key Next Steps" dataDxfId="100"/>
+    <tableColumn id="10" xr3:uid="{171C6211-BEA3-4026-BB75-96BBCCB9F34F}" name="Owners / Direct Responsible Individual" dataDxfId="99"/>
+    <tableColumn id="11" xr3:uid="{52ABC80D-1F46-4C95-ADD7-573DD9895B58}" name="Key Risks / Blockers" dataDxfId="98"/>
+    <tableColumn id="12" xr3:uid="{71A740DB-BF55-484E-83A5-FB5F077091BA}" name="Management Attention" dataDxfId="97"/>
+    <tableColumn id="13" xr3:uid="{0BB4D142-9FDE-40BF-863F-DB4D20B001FC}" name="Source / Notes" dataDxfId="96"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5124,19 +4926,19 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{4F3EA520-8DED-42FF-AE1D-EA325312A428}" name="TeamRoadmapTable66" displayName="TeamRoadmapTable66" ref="A1:M12" totalsRowShown="0">
   <autoFilter ref="A1:M12" xr:uid="{4F3EA520-8DED-42FF-AE1D-EA325312A428}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{BA6234AF-A2CE-4505-9800-89DF60D8D1B5}" name="#" dataDxfId="113"/>
-    <tableColumn id="2" xr3:uid="{0F3C72E8-FDF5-4C3E-8002-181B4941F0E2}" name="Project / Workstream" dataDxfId="112"/>
-    <tableColumn id="3" xr3:uid="{9BC4F7F1-CF84-4F48-8BFF-CF42E3B9F023}" name="Status" dataDxfId="111"/>
-    <tableColumn id="4" xr3:uid="{CA172084-5F14-449F-ADC0-E3442336F438}" name="Start Date" dataDxfId="110"/>
-    <tableColumn id="5" xr3:uid="{5775675D-FA3A-4EFF-BE16-EEEF395FE6EB}" name="Completion Date" dataDxfId="109"/>
-    <tableColumn id="6" xr3:uid="{B8FE331E-C500-40B6-A9EF-EA25F25C91DB}" name="% of Completion" dataDxfId="108"/>
-    <tableColumn id="7" xr3:uid="{1C903765-1ABA-47D7-8DCC-69299C6DC0EB}" name="Core Objective" dataDxfId="107"/>
-    <tableColumn id="8" xr3:uid="{D3FC52C0-445C-43EF-8AAE-45D8FB4561D6}" name="Current Progress" dataDxfId="106"/>
-    <tableColumn id="9" xr3:uid="{335B1F4D-C602-4F87-84FD-A1CFD3383BD6}" name="Key Next Steps" dataDxfId="105"/>
-    <tableColumn id="10" xr3:uid="{58EF9552-93B5-4FDF-B73F-68B923748B94}" name="Owners / Direct Responsible Individual" dataDxfId="104"/>
-    <tableColumn id="11" xr3:uid="{72675B8A-2AA3-4250-95A0-16DF36D3A611}" name="Key Risks / Blockers" dataDxfId="103"/>
-    <tableColumn id="12" xr3:uid="{CAC71F88-3105-4513-BA26-1DBF5CA737D2}" name="Management Attention" dataDxfId="102"/>
-    <tableColumn id="13" xr3:uid="{E603EA2D-4F37-4288-96B0-5ABDD9AF4C55}" name="Source / Notes" dataDxfId="101"/>
+    <tableColumn id="1" xr3:uid="{BA6234AF-A2CE-4505-9800-89DF60D8D1B5}" name="#" dataDxfId="95"/>
+    <tableColumn id="2" xr3:uid="{0F3C72E8-FDF5-4C3E-8002-181B4941F0E2}" name="Project / Workstream" dataDxfId="94"/>
+    <tableColumn id="3" xr3:uid="{9BC4F7F1-CF84-4F48-8BFF-CF42E3B9F023}" name="Status" dataDxfId="93"/>
+    <tableColumn id="4" xr3:uid="{CA172084-5F14-449F-ADC0-E3442336F438}" name="Start Date" dataDxfId="92"/>
+    <tableColumn id="5" xr3:uid="{5775675D-FA3A-4EFF-BE16-EEEF395FE6EB}" name="Completion Date" dataDxfId="91"/>
+    <tableColumn id="6" xr3:uid="{B8FE331E-C500-40B6-A9EF-EA25F25C91DB}" name="% of Completion" dataDxfId="90"/>
+    <tableColumn id="7" xr3:uid="{1C903765-1ABA-47D7-8DCC-69299C6DC0EB}" name="Core Objective" dataDxfId="89"/>
+    <tableColumn id="8" xr3:uid="{D3FC52C0-445C-43EF-8AAE-45D8FB4561D6}" name="Current Progress" dataDxfId="88"/>
+    <tableColumn id="9" xr3:uid="{335B1F4D-C602-4F87-84FD-A1CFD3383BD6}" name="Key Next Steps" dataDxfId="87"/>
+    <tableColumn id="10" xr3:uid="{58EF9552-93B5-4FDF-B73F-68B923748B94}" name="Owners / Direct Responsible Individual" dataDxfId="86"/>
+    <tableColumn id="11" xr3:uid="{72675B8A-2AA3-4250-95A0-16DF36D3A611}" name="Key Risks / Blockers" dataDxfId="85"/>
+    <tableColumn id="12" xr3:uid="{CAC71F88-3105-4513-BA26-1DBF5CA737D2}" name="Management Attention" dataDxfId="84"/>
+    <tableColumn id="13" xr3:uid="{E603EA2D-4F37-4288-96B0-5ABDD9AF4C55}" name="Source / Notes" dataDxfId="83"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5850,20 +5652,20 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C12">
-    <cfRule type="containsText" dxfId="100" priority="5" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="99" priority="6" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="98" priority="7" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="97" priority="8" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="82" priority="5" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="81" priority="6" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="80" priority="7" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="79" priority="8" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D4">
-    <cfRule type="containsText" dxfId="96" priority="13" operator="containsText" text="Red"/>
-    <cfRule type="containsText" dxfId="95" priority="14" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="94" priority="15" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="78" priority="13" operator="containsText" text="Red"/>
+    <cfRule type="containsText" dxfId="77" priority="14" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="76" priority="15" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D12">
-    <cfRule type="containsText" dxfId="93" priority="1" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="92" priority="2" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="91" priority="3" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="75" priority="1" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="74" priority="2" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="73" priority="3" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F7">
     <cfRule type="dataBar" priority="4">
@@ -6472,26 +6274,26 @@
       <c r="M11" s="99" t="s">
         <v>682</v>
       </c>
-      <c r="N11" s="114" t="s">
+      <c r="N11" s="112" t="s">
         <v>683</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2">
-    <cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="9" priority="6" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="7" priority="7" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="6" priority="8" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="72" priority="6" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="71" priority="5" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="70" priority="7" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="69" priority="8" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C8">
-    <cfRule type="containsText" dxfId="5" priority="11" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="4" priority="12" operator="containsText" text="Yellow"/>
-    <cfRule type="containsText" dxfId="3" priority="13" operator="containsText" text="Validation Pending"/>
+    <cfRule type="containsText" dxfId="68" priority="11" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="67" priority="12" operator="containsText" text="Yellow"/>
+    <cfRule type="containsText" dxfId="66" priority="13" operator="containsText" text="Validation Pending"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D8">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="65" priority="2" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="64" priority="3" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="63" priority="1" operator="containsText" text="At Risk"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F3">
     <cfRule type="dataBar" priority="4">
@@ -6508,6 +6310,13 @@
         <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
+    <cfRule type="dataBar" priority="40">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="min"/>
@@ -6515,6 +6324,13 @@
         <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
+    <cfRule type="dataBar" priority="36">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
     <cfRule type="dataBar" priority="16">
       <dataBar>
         <cfvo type="min"/>
@@ -6522,6 +6338,13 @@
         <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
+    <cfRule type="dataBar" priority="38">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
     <cfRule type="dataBar" priority="18">
       <dataBar>
         <cfvo type="min"/>
@@ -6529,84 +6352,14 @@
         <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
+    <cfRule type="dataBar" priority="42">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
     <cfRule type="dataBar" priority="20">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="22">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="24">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="26">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="28">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="30">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="32">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="34">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="36">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="38">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="40">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="42">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -6625,6 +6378,55 @@
         </ext>
       </extLst>
     </cfRule>
+    <cfRule type="dataBar" priority="22">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="28">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="24">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="26">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="30">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="32">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="34">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F8">
     <cfRule type="dataBar" priority="10">
@@ -6669,6 +6471,13 @@
         <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
+    <cfRule type="dataBar" priority="29">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
     <cfRule type="dataBar" priority="25">
       <dataBar>
         <cfvo type="min"/>
@@ -6676,6 +6485,41 @@
         <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
+    <cfRule type="dataBar" priority="37">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="31">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="39">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="35">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="41">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF5B9BD5"/>
+      </dataBar>
+    </cfRule>
     <cfRule type="dataBar" priority="27">
       <dataBar>
         <cfvo type="min"/>
@@ -6683,14 +6527,7 @@
         <color rgb="FF5B9BD5"/>
       </dataBar>
     </cfRule>
-    <cfRule type="dataBar" priority="29">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="31">
+    <cfRule type="dataBar" priority="43">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -6698,41 +6535,6 @@
       </dataBar>
     </cfRule>
     <cfRule type="dataBar" priority="33">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="35">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="37">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="39">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="41">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FF5B9BD5"/>
-      </dataBar>
-    </cfRule>
-    <cfRule type="dataBar" priority="43">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -6822,39 +6624,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="34" customHeight="1">
-      <c r="A1" s="112" t="s">
+      <c r="A1" s="113" t="s">
         <v>316</v>
       </c>
-      <c r="B1" s="112"/>
-      <c r="C1" s="112"/>
-      <c r="D1" s="112"/>
-      <c r="E1" s="112"/>
-      <c r="F1" s="112"/>
-      <c r="G1" s="112"/>
-      <c r="H1" s="112"/>
-      <c r="I1" s="112"/>
-      <c r="J1" s="112"/>
-      <c r="K1" s="112"/>
-      <c r="L1" s="112"/>
-      <c r="M1" s="112"/>
+      <c r="B1" s="113"/>
+      <c r="C1" s="113"/>
+      <c r="D1" s="113"/>
+      <c r="E1" s="113"/>
+      <c r="F1" s="113"/>
+      <c r="G1" s="113"/>
+      <c r="H1" s="113"/>
+      <c r="I1" s="113"/>
+      <c r="J1" s="113"/>
+      <c r="K1" s="113"/>
+      <c r="L1" s="113"/>
+      <c r="M1" s="113"/>
       <c r="N1" s="38"/>
     </row>
     <row r="2" spans="1:14" ht="46" customHeight="1">
-      <c r="A2" s="113" t="s">
+      <c r="A2" s="114" t="s">
         <v>317</v>
       </c>
-      <c r="B2" s="113"/>
-      <c r="C2" s="113"/>
-      <c r="D2" s="113"/>
-      <c r="E2" s="113"/>
-      <c r="F2" s="113"/>
-      <c r="G2" s="113"/>
-      <c r="H2" s="113"/>
-      <c r="I2" s="113"/>
-      <c r="J2" s="113"/>
-      <c r="K2" s="113"/>
-      <c r="L2" s="113"/>
-      <c r="M2" s="113"/>
+      <c r="B2" s="114"/>
+      <c r="C2" s="114"/>
+      <c r="D2" s="114"/>
+      <c r="E2" s="114"/>
+      <c r="F2" s="114"/>
+      <c r="G2" s="114"/>
+      <c r="H2" s="114"/>
+      <c r="I2" s="114"/>
+      <c r="J2" s="114"/>
+      <c r="K2" s="114"/>
+      <c r="L2" s="114"/>
+      <c r="M2" s="114"/>
       <c r="N2" s="39"/>
     </row>
     <row r="3" spans="1:14" ht="46" customHeight="1">
@@ -7125,58 +6927,58 @@
     <mergeCell ref="A2:M2"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:D7">
-    <cfRule type="expression" dxfId="72" priority="11">
+    <cfRule type="expression" dxfId="62" priority="11">
       <formula>OR(ISNUMBER(SEARCH("At Risk",C4)),ISNUMBER(SEARCH("Security Risk",C4)),ISNUMBER(SEARCH("Blocked",C4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="12">
+    <cfRule type="expression" dxfId="61" priority="12">
       <formula>OR(ISNUMBER(SEARCH("Green",C4)),ISNUMBER(SEARCH("Completed",C4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="70" priority="13">
+    <cfRule type="expression" dxfId="60" priority="13">
       <formula>AND(C4&lt;&gt;"",NOT(OR(ISNUMBER(SEARCH("At Risk",C4)),ISNUMBER(SEARCH("Security Risk",C4)),ISNUMBER(SEARCH("Blocked",C4)),ISNUMBER(SEARCH("Green",C4)),ISNUMBER(SEARCH("Completed",C4)))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8:D8">
-    <cfRule type="expression" dxfId="69" priority="1">
+    <cfRule type="expression" dxfId="59" priority="1">
       <formula>OR(ISNUMBER(SEARCH("At Risk",C8)),ISNUMBER(SEARCH("Security Risk",C8)),ISNUMBER(SEARCH("Blocked",C8)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="2">
+    <cfRule type="expression" dxfId="58" priority="2">
       <formula>OR(ISNUMBER(SEARCH("Green",C8)),ISNUMBER(SEARCH("Completed",C8)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="67" priority="3">
+    <cfRule type="expression" dxfId="57" priority="3">
       <formula>AND(C8&lt;&gt;"",NOT(OR(ISNUMBER(SEARCH("At Risk",C8)),ISNUMBER(SEARCH("Security Risk",C8)),ISNUMBER(SEARCH("Blocked",C8)),ISNUMBER(SEARCH("Green",C8)),ISNUMBER(SEARCH("Completed",C8)))))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H4:H7">
-    <cfRule type="containsText" dxfId="66" priority="14" operator="containsText" text="Completed">
+    <cfRule type="containsText" dxfId="56" priority="14" operator="containsText" text="Completed">
       <formula>NOT(ISERROR(SEARCH("Completed",H4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="65" priority="15" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="55" priority="15" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",H4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="64" priority="16" operator="containsText" text="At Risk">
+    <cfRule type="containsText" dxfId="54" priority="16" operator="containsText" text="At Risk">
       <formula>NOT(ISERROR(SEARCH("At Risk",H4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="63" priority="17" operator="containsText" text="Blocked">
+    <cfRule type="containsText" dxfId="53" priority="17" operator="containsText" text="Blocked">
       <formula>NOT(ISERROR(SEARCH("Blocked",H4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="62" priority="18" operator="containsText" text="Not Started">
+    <cfRule type="containsText" dxfId="52" priority="18" operator="containsText" text="Not Started">
       <formula>NOT(ISERROR(SEARCH("Not Started",H4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H8">
-    <cfRule type="containsText" dxfId="61" priority="4" operator="containsText" text="Completed">
+    <cfRule type="containsText" dxfId="51" priority="4" operator="containsText" text="Completed">
       <formula>NOT(ISERROR(SEARCH("Completed",H8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="60" priority="5" operator="containsText" text="In Progress">
+    <cfRule type="containsText" dxfId="50" priority="5" operator="containsText" text="In Progress">
       <formula>NOT(ISERROR(SEARCH("In Progress",H8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="59" priority="6" operator="containsText" text="At Risk">
+    <cfRule type="containsText" dxfId="49" priority="6" operator="containsText" text="At Risk">
       <formula>NOT(ISERROR(SEARCH("At Risk",H8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="58" priority="7" operator="containsText" text="Blocked">
+    <cfRule type="containsText" dxfId="48" priority="7" operator="containsText" text="Blocked">
       <formula>NOT(ISERROR(SEARCH("Blocked",H8)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="57" priority="8" operator="containsText" text="Not Started">
+    <cfRule type="containsText" dxfId="47" priority="8" operator="containsText" text="Not Started">
       <formula>NOT(ISERROR(SEARCH("Not Started",H8)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7900,10 +7702,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C10">
-    <cfRule type="containsText" dxfId="56" priority="2" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="55" priority="3" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="54" priority="4" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="53" priority="5" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="46" priority="2" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="45" priority="3" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="44" priority="4" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="43" priority="5" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="G2:G9">
     <cfRule type="dataBar" priority="8">
@@ -8465,20 +8267,20 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2">
-    <cfRule type="containsText" dxfId="52" priority="6" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="51" priority="5" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="50" priority="7" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="49" priority="8" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="42" priority="6" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="41" priority="5" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="40" priority="7" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="39" priority="8" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C8">
-    <cfRule type="containsText" dxfId="48" priority="11" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="47" priority="12" operator="containsText" text="Yellow"/>
-    <cfRule type="containsText" dxfId="46" priority="13" operator="containsText" text="Validation Pending"/>
+    <cfRule type="containsText" dxfId="38" priority="11" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="37" priority="12" operator="containsText" text="Yellow"/>
+    <cfRule type="containsText" dxfId="36" priority="13" operator="containsText" text="Validation Pending"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D8">
-    <cfRule type="containsText" dxfId="45" priority="2" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="44" priority="3" operator="containsText" text="Green"/>
-    <cfRule type="containsText" dxfId="43" priority="1" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="35" priority="2" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="34" priority="3" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="33" priority="1" operator="containsText" text="At Risk"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F3">
     <cfRule type="dataBar" priority="4">
@@ -9588,22 +9390,22 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B13">
-    <cfRule type="containsText" dxfId="42" priority="1" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="41" priority="2" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="40" priority="3" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="39" priority="4" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="32" priority="1" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="31" priority="2" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="30" priority="3" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="29" priority="4" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C13">
-    <cfRule type="containsText" dxfId="38" priority="6" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="37" priority="7" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="36" priority="9" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="28" priority="6" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="27" priority="7" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="26" priority="9" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:D13">
-    <cfRule type="containsText" dxfId="35" priority="8" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="25" priority="8" operator="containsText" text="At Risk"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D13">
-    <cfRule type="containsText" dxfId="34" priority="14" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="33" priority="15" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="24" priority="14" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="23" priority="15" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F12">
     <cfRule type="dataBar" priority="5">
@@ -10535,24 +10337,24 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="C11:C12">
-    <cfRule type="containsText" dxfId="32" priority="7" operator="containsText" text="Red"/>
-    <cfRule type="containsText" dxfId="31" priority="8" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="30" priority="9" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="22" priority="7" operator="containsText" text="Red"/>
+    <cfRule type="containsText" dxfId="21" priority="8" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="20" priority="9" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14:D15">
-    <cfRule type="containsText" dxfId="29" priority="4" operator="containsText" text="Red"/>
-    <cfRule type="containsText" dxfId="28" priority="5" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="27" priority="6" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="19" priority="4" operator="containsText" text="Red"/>
+    <cfRule type="containsText" dxfId="18" priority="5" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="17" priority="6" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C17:D17">
-    <cfRule type="containsText" dxfId="26" priority="1" operator="containsText" text="Red"/>
-    <cfRule type="containsText" dxfId="25" priority="2" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="24" priority="3" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="16" priority="1" operator="containsText" text="Red"/>
+    <cfRule type="containsText" dxfId="15" priority="2" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="14" priority="3" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D12">
-    <cfRule type="containsText" dxfId="23" priority="12" operator="containsText" text="Red"/>
-    <cfRule type="containsText" dxfId="22" priority="13" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="21" priority="14" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="13" priority="12" operator="containsText" text="Red"/>
+    <cfRule type="containsText" dxfId="12" priority="13" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="11" priority="14" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F13">
     <cfRule type="dataBar" priority="10">
@@ -11446,21 +11248,21 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B13:C13">
-    <cfRule type="containsText" dxfId="20" priority="1" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="19" priority="2" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="18" priority="3" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="17" priority="4" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="10" priority="1" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="8" priority="3" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="7" priority="4" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C12">
-    <cfRule type="containsText" dxfId="16" priority="6" operator="containsText" text="Completed"/>
-    <cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="In Progress"/>
-    <cfRule type="containsText" dxfId="14" priority="8" operator="containsText" text="At Risk"/>
-    <cfRule type="containsText" dxfId="13" priority="9" operator="containsText" text="Not Started"/>
+    <cfRule type="containsText" dxfId="6" priority="6" operator="containsText" text="Completed"/>
+    <cfRule type="containsText" dxfId="5" priority="7" operator="containsText" text="In Progress"/>
+    <cfRule type="containsText" dxfId="4" priority="8" operator="containsText" text="At Risk"/>
+    <cfRule type="containsText" dxfId="3" priority="9" operator="containsText" text="Not Started"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D13">
-    <cfRule type="containsText" dxfId="12" priority="14" operator="containsText" text="Red"/>
-    <cfRule type="containsText" dxfId="11" priority="15" operator="containsText" text="Amber"/>
-    <cfRule type="containsText" dxfId="10" priority="16" operator="containsText" text="Green"/>
+    <cfRule type="containsText" dxfId="2" priority="14" operator="containsText" text="Red"/>
+    <cfRule type="containsText" dxfId="1" priority="15" operator="containsText" text="Amber"/>
+    <cfRule type="containsText" dxfId="0" priority="16" operator="containsText" text="Green"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:F12">
     <cfRule type="dataBar" priority="5">

</xml_diff>